<commit_message>
OP analysis from the year 2007 to 2019
</commit_message>
<xml_diff>
--- a/results/HC_Extreme_Weeks_2019_upto9Dec_D5.xlsx
+++ b/results/HC_Extreme_Weeks_2019_upto9Dec_D5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UserA1\Documents\GitHub\Seismic_Amplitude_Timeseries_Analysis\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF6B5080-D269-4CF8-8836-39C34CC0AF30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EB524B4-5138-435F-A24A-CB441637DDCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="rsam_avg" sheetId="1" r:id="rId1"/>
@@ -1492,6 +1492,7 @@
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="2" width="23.44140625" customWidth="1"/>
     <col min="4" max="5" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>